<commit_message>
feat: august fleet reconciliation, legal accrual continuation, automatic vehicle availability, rental violation override, and cross-file duplicate payment guards
- Add 40+ supabase migrations/rollbacks: fleet report reconciliation, legal accrual continuation, vehicle custody corrections, payment classification dictionary, canonical duplicate payments views, active revenue payments view, automatic vehicle availability enforcement, rental violation override
- Add RentalViolationOverrideContext and vehicleOperationalStatus utilities
- Harden legal claim sources, taqadi narrative, legal memo requests, and document generator
- Fix vehicle financial trigger recursion and contract creation with unpaid violations
- Update dashboard stats, finance hub, quick payment recording, and contract wizards
- Add migration tests and design docs
</commit_message>
<xml_diff>
--- a/اسماء-عقود-سطح-المكتب.xlsx
+++ b/اسماء-عقود-سطح-المكتب.xlsx
@@ -2987,7 +2987,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>أيمن خليفة حمادي</t>
+          <t>ايمن خليفة حمادي</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -3038,7 +3038,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>أيمن خليفة حمادي</t>
+          <t>ايمن خليفة حمادي</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -5568,7 +5568,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>حمزة البشير يانس</t>
+          <t>حمد البشير يانس</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5619,7 +5619,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>حمزة البشير يانس</t>
+          <t>حمد البشير يانس</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -15149,7 +15149,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>أيمن خليفة حمادي</t>
+          <t>ايمن خليفة حمادي</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -16445,7 +16445,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>حمزة البشير يانس</t>
+          <t>حمد البشير يانس</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -19491,7 +19491,6 @@
           <t>21860</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>محمد العويني.pdf</t>

</xml_diff>